<commit_message>
Add Power BI raw-vs-modeled eval reports (PBIR) + blank eval template
Hand-author two PBIR reports, one page per eval question (12 each):
- modeled report (MultiSource_Modeled) answers all 12 via the governed measures
- raw report (MultiSource_Raw) is an honest demo: implicit aggregations on real
  columns only, exposing the planted traps (no revenue column, free-text/ITM
  joins, text dates, missing referential integrity). No report-level measures.

pbip/build_reports.py is the deterministic generator for both. Also blank the
tracked eval workbook to a reusable template (questions + gold kept, run
comments/scores cleared) and git-ignore the filled results copy + PBIR
per-user localSettings.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval/MultiSourceAgent_Eval.xlsx
+++ b/eval/MultiSourceAgent_Eval.xlsx
@@ -2,19 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-3765" windowWidth="38640" windowHeight="21840" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Eval" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Conventions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eval'!$A$2:$P$14</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -23,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -33,23 +30,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <charset val="1"/>
-      <family val="0"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
@@ -57,29 +38,16 @@
     <font>
       <name val="Arial"/>
       <charset val="1"/>
-      <family val="0"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <family val="0"/>
-      <i val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <family val="0"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -94,34 +62,46 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="FF2E5496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4EC"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4EC"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <fgColor theme="6" tint="0.5999938962981048"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5496"/>
+        <fgColor theme="9" tint="0.5999938962981048"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor theme="5" tint="0.5999938962981048"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.7999816888943144"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -145,109 +125,129 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="20">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="25">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
-    <cellStyle name="Currency" xfId="3" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
-    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -306,47 +306,55 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E79"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -354,12 +362,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -388,7 +396,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -409,7 +417,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -460,7 +468,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -478,11 +486,13 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -492,618 +502,541 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" style="14" min="1" max="1"/>
-    <col width="5" customWidth="1" style="14" min="2" max="2"/>
-    <col width="34" customWidth="1" style="14" min="3" max="3"/>
-    <col width="30" customWidth="1" style="14" min="4" max="4"/>
-    <col width="40" customWidth="1" style="14" min="5" max="5"/>
-    <col width="34" customWidth="1" style="14" min="6" max="6"/>
-    <col width="30" customWidth="1" style="14" min="7" max="7"/>
-    <col width="7" customWidth="1" style="14" min="8" max="8"/>
-    <col width="11" customWidth="1" style="14" min="9" max="9"/>
-    <col width="30" customWidth="1" style="14" min="10" max="10"/>
-    <col width="7" customWidth="1" style="14" min="11" max="11"/>
-    <col width="11" customWidth="1" style="14" min="12" max="12"/>
-    <col width="30" customWidth="1" style="14" min="13" max="13"/>
-    <col width="7" customWidth="1" style="14" min="14" max="14"/>
-    <col width="11" customWidth="1" style="14" min="15" max="15"/>
-    <col width="26" customWidth="1" style="14" min="16" max="16"/>
+    <col width="4.42578125" bestFit="1" customWidth="1" style="9" min="1" max="2"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="9" min="3" max="3"/>
+    <col width="30" customWidth="1" style="9" min="4" max="4"/>
+    <col width="64.42578125" customWidth="1" style="9" min="5" max="5"/>
+    <col width="34" customWidth="1" style="9" min="6" max="6"/>
+    <col width="45.42578125" customWidth="1" style="15" min="7" max="7"/>
+    <col width="15.28515625" customWidth="1" style="9" min="8" max="8"/>
+    <col width="45.42578125" customWidth="1" style="15" min="9" max="9"/>
+    <col width="15.28515625" customWidth="1" style="9" min="10" max="10"/>
+    <col width="45.42578125" customWidth="1" style="15" min="11" max="11"/>
+    <col width="15.28515625" customWidth="1" style="9" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>What it tests</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>Gold answer</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>Expected Raw (bare) failure</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>Raw (bare)</t>
         </is>
       </c>
-      <c r="H1" s="15" t="n"/>
-      <c r="I1" s="15" t="n"/>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="H1" s="18" t="n"/>
+      <c r="I1" s="10" t="inlineStr">
         <is>
           <t>Raw_Plus</t>
         </is>
       </c>
-      <c r="K1" s="15" t="n"/>
-      <c r="L1" s="15" t="n"/>
-      <c r="M1" s="15" t="inlineStr">
+      <c r="J1" s="18" t="n"/>
+      <c r="K1" s="10" t="inlineStr">
         <is>
           <t>Modeled</t>
         </is>
       </c>
-      <c r="N1" s="15" t="n"/>
-      <c r="O1" s="15" t="n"/>
-      <c r="P1" s="15" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="L1" s="18" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="n"/>
-      <c r="B2" s="16" t="n"/>
-      <c r="C2" s="16" t="n"/>
-      <c r="D2" s="16" t="n"/>
-      <c r="E2" s="16" t="n"/>
-      <c r="F2" s="16" t="n"/>
-      <c r="G2" s="16" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-      <c r="H2" s="16" t="inlineStr">
+      <c r="A2" s="19" t="n"/>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="n"/>
+      <c r="F2" s="19" t="n"/>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="I2" s="16" t="inlineStr">
-        <is>
-          <t>Tokens/CUs</t>
-        </is>
-      </c>
-      <c r="J2" s="16" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-      <c r="K2" s="16" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="L2" s="16" t="inlineStr">
-        <is>
-          <t>Tokens/CUs</t>
-        </is>
-      </c>
-      <c r="M2" s="16" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-      <c r="N2" s="16" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="O2" s="16" t="inlineStr">
-        <is>
-          <t>Tokens/CUs</t>
-        </is>
-      </c>
-      <c r="P2" s="16" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+    </row>
+    <row r="3" ht="30" customHeight="1" s="9">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="B3" s="18" t="n">
+      <c r="B3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>What was our revenue in Q1 2026 by channel?</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Both answer; baseline for token comparison</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Online $7.030M / Retail $7.156M / Wholesale $6.911M; total $21.097M (ERP, Jan-Mar 2026)</t>
         </is>
       </c>
-      <c r="F3" s="19" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Should pass — single clean table</t>
         </is>
       </c>
-      <c r="G3" s="17" t="n"/>
-      <c r="H3" s="18" t="n"/>
-      <c r="I3" s="17" t="n"/>
-      <c r="J3" s="17" t="n"/>
-      <c r="K3" s="18" t="n"/>
-      <c r="L3" s="17" t="n"/>
-      <c r="M3" s="17" t="n"/>
-      <c r="N3" s="18" t="n"/>
-      <c r="O3" s="17" t="n"/>
-      <c r="P3" s="17" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="12" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="12" t="n"/>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="12" t="n"/>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="9">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>What are our top 5 products by revenue?</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>May differ if it tries to include unjoinable sources</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>SKU-0074 Terminal Block $6.68M; SKU-0094 Hydraulic Hose $4.86M; SKU-0014 Rocker Switch $4.77M; SKU-0079 IEC Connector $4.42M; SKU-0080 Stretch Wrap $4.33M (ERP, full window)</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Should pass</t>
         </is>
       </c>
-      <c r="G4" s="17" t="n"/>
-      <c r="H4" s="18" t="n"/>
-      <c r="I4" s="17" t="n"/>
-      <c r="J4" s="17" t="n"/>
-      <c r="K4" s="18" t="n"/>
-      <c r="L4" s="17" t="n"/>
-      <c r="M4" s="17" t="n"/>
-      <c r="N4" s="18" t="n"/>
-      <c r="O4" s="17" t="n"/>
-      <c r="P4" s="17" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="12" t="n"/>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="12" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="9">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>What was our stockout rate in May 2026?</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Definition drift possible (share of SKUs vs share of rows)</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>1.52% of SKU-location-days (ERP daily snapshots, May 2026)</t>
         </is>
       </c>
-      <c r="F5" s="19" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Should pass — is_stockout flag exists raw</t>
         </is>
       </c>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="18" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="18" t="n"/>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="18" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="17" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="12" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="12" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="105" customHeight="1" s="9">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>What were total company sales in May 2026, including Lakeside and the marketplace?</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Tests cross-source conformance + gross/net rule</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>$10.054M = ERP $8.382M + marketplace NET $0.622M + Lakeside $1.051M</t>
         </is>
       </c>
-      <c r="F6" s="19" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>ERP-only $8.382M, or $9.106M using marketplace GROSS; Lakeside missed (text DD/MM/YYYY dates, no join)</t>
         </is>
       </c>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="18" t="n"/>
-      <c r="I6" s="17" t="n"/>
-      <c r="J6" s="17" t="n"/>
-      <c r="K6" s="18" t="n"/>
-      <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="18" t="n"/>
-      <c r="O6" s="17" t="n"/>
-      <c r="P6" s="17" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="14" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="13" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="12" t="n"/>
+    </row>
+    <row r="7" ht="105" customHeight="1" s="9">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Q5</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>What is our net marketplace revenue after fees, by month?</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Gross-vs-net trap</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Full window $7.335M net (gross $8.534M, fees 14.0%). E.g. Mar-26 $638K, Apr-26 $594K, May-26 $622K</t>
         </is>
       </c>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Reports gross from mm_orders (no settlement join): ~16% overstated</t>
         </is>
       </c>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="18" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="18" t="n"/>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="18" t="n"/>
-      <c r="O7" s="17" t="n"/>
-      <c r="P7" s="17" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="14" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="14" t="n"/>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="12" t="n"/>
+    </row>
+    <row r="8" ht="75" customHeight="1" s="9">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Q6</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Which products generate the most helpdesk tickets per 1,000 units sold?</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Free-text conformance + ratio convention</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>SKU-0045 Titan Solenoid Valve 142.7/1K (2,041 tickets); SKU-0014 Titan Rocker Switch 115.9/1K (1,967); next SKU-0085 at 40.5. Convention: SKUs with &gt;=1,000 units; 88% of ticket refs resolve</t>
         </is>
       </c>
-      <c r="F8" s="19" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Cannot join free-text productRef to units; hallucinated join or refusal</t>
         </is>
       </c>
-      <c r="G8" s="17" t="n"/>
-      <c r="H8" s="18" t="n"/>
-      <c r="I8" s="17" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="6" t="n"/>
       <c r="J8" s="17" t="n"/>
-      <c r="K8" s="18" t="n"/>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="17" t="n"/>
-      <c r="N8" s="18" t="n"/>
-      <c r="O8" s="17" t="n"/>
-      <c r="P8" s="17" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="12" t="n"/>
+    </row>
+    <row r="9" ht="90" customHeight="1" s="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Q7</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>What is the service parts attach rate for Hydraulics products?</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>ITM code conformance</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>8.1 parts per 100 units sold (16,156 parts / 199,192 Hydraulics units)</t>
         </is>
       </c>
-      <c r="F9" s="19" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Cannot resolve ITM- codes to SKUs; wrong denominator or hallucination</t>
         </is>
       </c>
-      <c r="G9" s="17" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="17" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="16" t="n"/>
+      <c r="I9" s="6" t="n"/>
       <c r="J9" s="17" t="n"/>
-      <c r="K9" s="18" t="n"/>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="17" t="n"/>
-      <c r="N9" s="18" t="n"/>
-      <c r="O9" s="17" t="n"/>
-      <c r="P9" s="17" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="13" t="n"/>
+    </row>
+    <row r="10" ht="105" customHeight="1" s="9">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Which A-class products have open complaints AND are at stockout risk in the merged network?</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>The flagship multi-hop question</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>SKU-0014 Titan Rocker Switch 20A and SKU-0045 Titan Solenoid Valve 1in (open complaint tickets; on-hand &lt;= safety stock at 2026-05-31; near-zero Lakeside counts)</t>
         </is>
       </c>
-      <c r="F10" s="19" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Multi-hop across 4 sources fails; likely hallucinated list</t>
         </is>
       </c>
-      <c r="G10" s="17" t="n"/>
-      <c r="H10" s="18" t="n"/>
-      <c r="I10" s="17" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="6" t="n"/>
       <c r="J10" s="17" t="n"/>
-      <c r="K10" s="18" t="n"/>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="17" t="n"/>
-      <c r="N10" s="18" t="n"/>
-      <c r="O10" s="17" t="n"/>
-      <c r="P10" s="17" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="12" t="n"/>
+    </row>
+    <row r="11" ht="90" customHeight="1" s="9">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Q9</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Compare Lakeside store sell-through vs our DCs since the acquisition.</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Mixed-grain inventory + acquisition date</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Feb-May 2026: Lakeside 2.85x (46,145 units / 16,187 avg on-hand) vs DCs 1.70x (234,391 / 138,261). Lakeside turns ~1.7x faster</t>
         </is>
       </c>
-      <c r="F11" s="19" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Cannot parse Lakeside text dates or weekly counts; no answer or invented numbers</t>
         </is>
       </c>
-      <c r="G11" s="17" t="n"/>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="17" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="6" t="n"/>
       <c r="J11" s="17" t="n"/>
-      <c r="K11" s="18" t="n"/>
-      <c r="L11" s="17" t="n"/>
-      <c r="M11" s="17" t="n"/>
-      <c r="N11" s="18" t="n"/>
-      <c r="O11" s="17" t="n"/>
-      <c r="P11" s="17" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="12" t="n"/>
+    </row>
+    <row r="12" ht="75" customHeight="1" s="9">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Q10</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>What were Lakeside sales on 03/02/2026?</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Date-format trap</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>$36,836 (Feb 3, 2026 — dates are DD/MM/YYYY). An MM/DD misparse gives Mar 2 = $44,972</t>
         </is>
       </c>
-      <c r="F12" s="19" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Misparses as March 2 or fails on text date</t>
         </is>
       </c>
-      <c r="G12" s="17" t="n"/>
-      <c r="H12" s="18" t="n"/>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="17" t="n"/>
-      <c r="K12" s="18" t="n"/>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="17" t="n"/>
-      <c r="N12" s="18" t="n"/>
-      <c r="O12" s="17" t="n"/>
-      <c r="P12" s="17" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="13" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="12" t="n"/>
+    </row>
+    <row r="13" ht="75" customHeight="1" s="9">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Q11</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>How much revenue has Lakeside generated since the acquisition?</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Period convention from Prep-for-AI</t>
         </is>
       </c>
-      <c r="E13" s="19" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>$4.324M (Feb 1 - May 31, 2026; ~9% from Lakeside store-brand items)</t>
         </is>
       </c>
-      <c r="F13" s="19" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>No acquisition date knowledge + text dates: wrong period or no answer</t>
         </is>
       </c>
-      <c r="G13" s="17" t="n"/>
-      <c r="H13" s="18" t="n"/>
-      <c r="I13" s="17" t="n"/>
-      <c r="J13" s="17" t="n"/>
-      <c r="K13" s="18" t="n"/>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="17" t="n"/>
-      <c r="N13" s="18" t="n"/>
-      <c r="O13" s="17" t="n"/>
-      <c r="P13" s="17" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="17" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="90" customHeight="1" s="9">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Q12</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>How much marketplace revenue can't be tied to one of our products?</t>
         </is>
       </c>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Data-quality awareness question</t>
         </is>
       </c>
-      <c r="E14" s="19" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>$94K gross (1.1% of marketplace gross) from ~10 stale/unmapped listings</t>
         </is>
       </c>
-      <c r="F14" s="19" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>No xref join: either 0% or everything unmapped</t>
         </is>
       </c>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="18" t="n"/>
-      <c r="I14" s="17" t="n"/>
-      <c r="J14" s="17" t="n"/>
-      <c r="K14" s="18" t="n"/>
-      <c r="L14" s="17" t="n"/>
-      <c r="M14" s="17" t="n"/>
-      <c r="N14" s="18" t="n"/>
-      <c r="O14" s="17" t="n"/>
-      <c r="P14" s="17" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="16" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1120,19 +1053,17 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:P14"/>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="A16:F16"/>
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="A17:P17"/>
-    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="K1:L1"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A17:L17"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:F2"/>
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="I1:J1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1145,217 +1076,199 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="14" min="1" max="1"/>
-    <col width="42" customWidth="1" style="14" min="2" max="2"/>
-    <col width="11" customWidth="1" style="14" min="3" max="3"/>
-    <col width="6" customWidth="1" style="14" min="4" max="4"/>
-    <col width="9" customWidth="1" style="14" min="5" max="5"/>
-    <col width="11" customWidth="1" style="14" min="6" max="6"/>
-    <col width="11" customWidth="1" style="14" min="7" max="7"/>
-    <col width="10" customWidth="1" style="14" min="8" max="8"/>
-    <col width="15" customWidth="1" style="14" min="9" max="9"/>
-    <col width="10" customWidth="1" style="14" min="10" max="10"/>
-    <col width="13" customWidth="1" style="14" min="11" max="11"/>
+    <col width="22.140625" bestFit="1" customWidth="1" style="9" min="1" max="1"/>
+    <col width="52.85546875" bestFit="1" customWidth="1" style="9" min="2" max="2"/>
+    <col width="10.5703125" bestFit="1" customWidth="1" style="9" min="3" max="3"/>
+    <col width="4.85546875" bestFit="1" customWidth="1" style="9" min="4" max="4"/>
+    <col width="9" customWidth="1" style="9" min="5" max="5"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" style="9" min="6" max="6"/>
+    <col width="9.5703125" bestFit="1" customWidth="1" style="9" min="7" max="7"/>
+    <col width="9.85546875" bestFit="1" customWidth="1" style="9" min="8" max="8"/>
+    <col width="15.85546875" bestFit="1" customWidth="1" style="9" min="9" max="9"/>
+    <col width="10" customWidth="1" style="9" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Agent</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Data source</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Total score</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Max</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>% of max</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Correct (2)</t>
         </is>
       </c>
-      <c r="G1" s="16" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Partial (1)</t>
         </is>
       </c>
-      <c r="H1" s="16" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Wrong (0)</t>
         </is>
       </c>
-      <c r="I1" s="16" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Hallucinated (-1)</t>
         </is>
       </c>
-      <c r="J1" s="16" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="K1" s="16" t="inlineStr">
-        <is>
-          <t>Avg tokens/CUs</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>SupplyAgent_Raw</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>MultiSource_Raw model — no instructions</t>
         </is>
       </c>
-      <c r="C2" s="20">
+      <c r="C2" s="7">
         <f>SUM(Eval!H3:H14)</f>
         <v/>
       </c>
-      <c r="D2" s="20" t="n">
+      <c r="D2" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="E2" s="21">
+      <c r="E2" s="8">
         <f>IFERROR(C2/D2,0)</f>
         <v/>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="7">
         <f>COUNTIF(Eval!H3:H14,2)</f>
         <v/>
       </c>
-      <c r="G2" s="20">
+      <c r="G2" s="7">
         <f>COUNTIF(Eval!H3:H14,1)</f>
         <v/>
       </c>
-      <c r="H2" s="20">
+      <c r="H2" s="7">
         <f>COUNTIF(Eval!H3:H14,0)</f>
         <v/>
       </c>
-      <c r="I2" s="20">
+      <c r="I2" s="7">
         <f>COUNTIF(Eval!H3:H14,-1)</f>
         <v/>
       </c>
-      <c r="J2" s="20">
+      <c r="J2" s="7">
         <f>COUNT(Eval!H3:H14)</f>
         <v/>
       </c>
-      <c r="K2" s="20">
-        <f>IFERROR(AVERAGE(Eval!I3:I14),0)</f>
-        <v/>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>SupplyAgent_Raw_Plus</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>lh_supply_demo SQL endpoint + heavy agent instructions</t>
         </is>
       </c>
-      <c r="C3" s="20">
-        <f>SUM(Eval!K3:K14)</f>
-        <v/>
-      </c>
-      <c r="D3" s="20" t="n">
+      <c r="C3" s="7">
+        <f>SUM(Eval!J3:J14)</f>
+        <v/>
+      </c>
+      <c r="D3" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="E3" s="21">
+      <c r="E3" s="8">
         <f>IFERROR(C3/D3,0)</f>
         <v/>
       </c>
-      <c r="F3" s="20">
-        <f>COUNTIF(Eval!K3:K14,2)</f>
-        <v/>
-      </c>
-      <c r="G3" s="20">
-        <f>COUNTIF(Eval!K3:K14,1)</f>
-        <v/>
-      </c>
-      <c r="H3" s="20">
-        <f>COUNTIF(Eval!K3:K14,0)</f>
-        <v/>
-      </c>
-      <c r="I3" s="20">
-        <f>COUNTIF(Eval!K3:K14,-1)</f>
-        <v/>
-      </c>
-      <c r="J3" s="20">
-        <f>COUNT(Eval!K3:K14)</f>
-        <v/>
-      </c>
-      <c r="K3" s="20">
-        <f>IFERROR(AVERAGE(Eval!L3:L14),0)</f>
+      <c r="F3" s="7">
+        <f>COUNTIF(Eval!J3:J14,2)</f>
+        <v/>
+      </c>
+      <c r="G3" s="7">
+        <f>COUNTIF(Eval!J3:J14,1)</f>
+        <v/>
+      </c>
+      <c r="H3" s="7">
+        <f>COUNTIF(Eval!J3:J14,0)</f>
+        <v/>
+      </c>
+      <c r="I3" s="7">
+        <f>COUNTIF(Eval!J3:J14,-1)</f>
+        <v/>
+      </c>
+      <c r="J3" s="7">
+        <f>COUNT(Eval!J3:J14)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>SupplyAgent_Modeled</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>MultiSource_Modeled star + Prep-for-AI</t>
         </is>
       </c>
-      <c r="C4" s="20">
-        <f>SUM(Eval!N3:N14)</f>
-        <v/>
-      </c>
-      <c r="D4" s="20" t="n">
+      <c r="C4" s="7">
+        <f>SUM(Eval!L3:L14)</f>
+        <v/>
+      </c>
+      <c r="D4" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="E4" s="21">
+      <c r="E4" s="8">
         <f>IFERROR(C4/D4,0)</f>
         <v/>
       </c>
-      <c r="F4" s="20">
-        <f>COUNTIF(Eval!N3:N14,2)</f>
-        <v/>
-      </c>
-      <c r="G4" s="20">
-        <f>COUNTIF(Eval!N3:N14,1)</f>
-        <v/>
-      </c>
-      <c r="H4" s="20">
-        <f>COUNTIF(Eval!N3:N14,0)</f>
-        <v/>
-      </c>
-      <c r="I4" s="20">
-        <f>COUNTIF(Eval!N3:N14,-1)</f>
-        <v/>
-      </c>
-      <c r="J4" s="20">
-        <f>COUNT(Eval!N3:N14)</f>
-        <v/>
-      </c>
-      <c r="K4" s="20">
-        <f>IFERROR(AVERAGE(Eval!O3:O14),0)</f>
+      <c r="F4" s="7">
+        <f>COUNTIF(Eval!L3:L14,2)</f>
+        <v/>
+      </c>
+      <c r="G4" s="7">
+        <f>COUNTIF(Eval!L3:L14,1)</f>
+        <v/>
+      </c>
+      <c r="H4" s="7">
+        <f>COUNTIF(Eval!L3:L14,0)</f>
+        <v/>
+      </c>
+      <c r="I4" s="7">
+        <f>COUNTIF(Eval!L3:L14,-1)</f>
+        <v/>
+      </c>
+      <c r="J4" s="7">
+        <f>COUNT(Eval!L3:L14)</f>
         <v/>
       </c>
     </row>
@@ -1366,164 +1279,163 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" style="22" min="1" max="1"/>
-    <col width="80" customWidth="1" style="22" min="2" max="2"/>
+    <col width="23.85546875" bestFit="1" customWidth="1" style="9" min="1" max="1"/>
+    <col width="80.7109375" bestFit="1" customWidth="1" style="9" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="14">
-      <c r="A1" s="23" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="9">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Convention</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="14">
-      <c r="A2" s="24" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="9">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Data window</t>
         </is>
       </c>
-      <c r="B2" s="24" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2025-06-01 to 2026-05-31</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="14">
-      <c r="A3" s="24" t="inlineStr">
+    <row r="3" ht="15" customHeight="1" s="9">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Acquisition date (Lakeside)</t>
         </is>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>2026-02-01</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="14">
-      <c r="A4" s="24" t="inlineStr">
+    <row r="4" ht="15" customHeight="1" s="9">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>'Total / company sales'</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>ERP + marketplace NET + Lakeside</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="14">
-      <c r="A5" s="24" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="9">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Marketplace revenue</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>NET of fees (payoutAmount) unless 'gross' is asked</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="14">
-      <c r="A6" s="24" t="inlineStr">
+    <row r="6" ht="15" customHeight="1" s="9">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Lakeside dates</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>TEXT DD/MM/YYYY in raw exports</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="14">
-      <c r="A7" s="24" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="9">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Stockout rate</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>share of SKU-location-day snapshots with is_stockout = 1</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="14">
-      <c r="A8" s="24" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="9">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Stockout risk</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>on-hand &lt;= safety stock at latest snapshot (ERP) or near-zero latest weekly count (Lakeside)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="14">
-      <c r="A9" s="24" t="inlineStr">
+    <row r="9" ht="15" customHeight="1" s="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Complaint</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>helpdesk categoryId = 1 (Product complaint)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="14">
-      <c r="A10" s="24" t="inlineStr">
+    <row r="10" ht="15" customHeight="1" s="9">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Tickets per 1K units</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>resolved product refs only (88%); SKUs with &gt;= 1,000 units sold</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="14">
-      <c r="A11" s="24" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="9">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Sell-through ratio</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>units sold / average on-hand units over the period</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="14">
-      <c r="A12" s="24" t="inlineStr">
+    <row r="12" ht="15" customHeight="1" s="9">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Token/CU measurement</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Capacity Metrics app (capacity admin on fabricassesmentcoe) or Foundry/SDK</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>